<commit_message>
chore(templates): nota sobre coluna Estado no Registo de Riscos
Passo 3 das instruções explicita que o cliente preenche a coluna
Estado (Em curso/Concluído/Transferido) e que o Painel de Controlo
se atualiza a partir dela — "0 riscos tratados" é normal até preencher.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/assets/templates/registo-riscos.xlsx
+++ b/backend/assets/templates/registo-riscos.xlsx
@@ -58,7 +58,7 @@
     <t xml:space="preserve">2. Acrescente riscos que o scan não deteta (ex.: falhas de processo, fornecedores, pessoas) em linhas novas, marcando a coluna Origem como "Manual"</t>
   </si>
   <si>
-    <t xml:space="preserve">3. Preencha o Responsável de cada risco e atualize o Estado à medida que as medidas de tratamento são aplicadas</t>
+    <t xml:space="preserve">3. Preencha, para cada risco: o RESPONSÁVEL (quem trata) e o ESTADO na coluna "Estado" (Em curso / Concluído / Transferido). O Painel de Controlo atualiza-se automaticamente a partir desta coluna — enquanto não a preencher, o Painel mostra 0 riscos tratados (é normal).</t>
   </si>
   <si>
     <t xml:space="preserve">4. O Nível de Risco é calculado automaticamente (Probabilidade × Impacto) — não precisa de o preencher</t>
@@ -977,7 +977,7 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="11" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="11" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -989,7 +989,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="12" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="12" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1001,7 +1001,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="13" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="13" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1013,7 +1013,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="14" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>

</xml_diff>